<commit_message>
changes done in java 50
</commit_message>
<xml_diff>
--- a/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
+++ b/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
@@ -4,24 +4,25 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="6" r:id="rId4"/>
+    <sheet name="Sheet4" sheetId="7" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet3!$A$1:$G$199</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Sheet5!$A$1:$F$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Sheet5!$A$1:$F$200</definedName>
   </definedNames>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2702" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2726" uniqueCount="517">
   <si>
     <t>Category</t>
   </si>
@@ -1566,6 +1567,12 @@
   </si>
   <si>
     <t>Complete</t>
+  </si>
+  <si>
+    <t>https://www.naukri.com/job-listings-java-lead-talworx-solutions-thane-mumbai-all-areas-9-to-12-years-230426015400?src=jobsearchDesk&amp;sid=17790218769593763&amp;xp=1&amp;px=1</t>
+  </si>
+  <si>
+    <t>https://wissen.zohorecruit.in/jobs/Careers/80238000057776296/Java-Lead?source=LinkedIn-Premium&amp;embedsource=LinkedIn%2BLimited%2BListings</t>
   </si>
 </sst>
 </file>
@@ -1648,7 +1655,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1680,6 +1687,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10316,6 +10326,9 @@
       <c r="E19" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F19" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
@@ -10333,6 +10346,9 @@
       <c r="E20" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F20" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -10350,6 +10366,9 @@
       <c r="E21" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F21" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
@@ -10367,6 +10386,9 @@
       <c r="E22" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F22" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
@@ -10384,6 +10406,9 @@
       <c r="E23" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F23" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
@@ -10401,6 +10426,9 @@
       <c r="E24" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F24" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -10418,6 +10446,9 @@
       <c r="E25" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F25" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
@@ -10435,6 +10466,9 @@
       <c r="E26" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F26" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -10452,6 +10486,9 @@
       <c r="E27" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F27" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
@@ -10469,6 +10506,9 @@
       <c r="E28" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F28" s="12" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
@@ -10538,7 +10578,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -10555,7 +10595,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -10572,7 +10612,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -10589,7 +10629,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -10606,7 +10646,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -10622,8 +10662,11 @@
       <c r="E37" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -10639,8 +10682,11 @@
       <c r="E38" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -10656,8 +10702,11 @@
       <c r="E39" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -10673,8 +10722,11 @@
       <c r="E40" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F40" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -10688,10 +10740,13 @@
         <v>158</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+      <c r="F41" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -10708,7 +10763,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -10725,7 +10780,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -10742,7 +10797,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -10759,7 +10814,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -10776,7 +10831,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -10793,7 +10848,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -10827,7 +10882,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -10841,10 +10896,10 @@
         <v>181</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -10858,7 +10913,7 @@
         <v>183</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -11082,7 +11137,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -11099,7 +11154,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -11116,7 +11171,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -11133,7 +11188,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -11149,8 +11204,11 @@
       <c r="E68" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F68" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -11166,8 +11224,11 @@
       <c r="E69" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -11183,8 +11244,11 @@
       <c r="E70" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F70" s="12" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -11201,7 +11265,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -11218,7 +11282,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -11235,7 +11299,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -11252,7 +11316,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -11269,7 +11333,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -11286,7 +11350,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -11303,7 +11367,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -11317,10 +11381,10 @@
         <v>134</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -11337,7 +11401,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -12170,7 +12234,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>128</v>
       </c>
@@ -12184,10 +12248,10 @@
         <v>324</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>129</v>
       </c>
@@ -12201,10 +12265,10 @@
         <v>70</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>130</v>
       </c>
@@ -12218,7 +12282,7 @@
         <v>327</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
@@ -12235,7 +12299,7 @@
         <v>329</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
@@ -13377,6 +13441,23 @@
         <v>457</v>
       </c>
     </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" s="1">
+        <v>199</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C200" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D200" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E200" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B205" s="11" t="s">
         <v>511</v>
@@ -13393,7 +13474,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F199">
+  <autoFilter ref="A1:F200">
     <filterColumn colId="4">
       <filters>
         <filter val="P1"/>
@@ -13403,4 +13484,27 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="87.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>516</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added new features in overjava 50 and maximum 200k java8
</commit_message>
<xml_diff>
--- a/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
+++ b/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2726" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2737" uniqueCount="517">
   <si>
     <t>Category</t>
   </si>
@@ -1686,9 +1686,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9977,7 +9979,7 @@
     <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" style="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9996,6 +9998,9 @@
       <c r="E1" s="10" t="s">
         <v>454</v>
       </c>
+      <c r="F1" s="10" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
@@ -10013,6 +10018,7 @@
       <c r="E2" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
@@ -10030,6 +10036,7 @@
       <c r="E3" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
@@ -10047,6 +10054,7 @@
       <c r="E4" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -10064,6 +10072,7 @@
       <c r="E5" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -10081,6 +10090,7 @@
       <c r="E6" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -10098,6 +10108,7 @@
       <c r="E7" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -10115,6 +10126,7 @@
       <c r="E8" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -10132,7 +10144,7 @@
       <c r="E9" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10152,7 +10164,7 @@
       <c r="E10" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10172,6 +10184,7 @@
       <c r="E11" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -10189,7 +10202,7 @@
       <c r="E12" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10209,7 +10222,7 @@
       <c r="E13" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10229,7 +10242,7 @@
       <c r="E14" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10249,6 +10262,7 @@
       <c r="E15" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -10266,7 +10280,7 @@
       <c r="E16" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10286,7 +10300,7 @@
       <c r="E17" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10306,7 +10320,7 @@
       <c r="E18" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10326,7 +10340,7 @@
       <c r="E19" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10346,7 +10360,7 @@
       <c r="E20" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10366,7 +10380,7 @@
       <c r="E21" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10386,7 +10400,7 @@
       <c r="E22" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10406,7 +10420,7 @@
       <c r="E23" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10426,7 +10440,7 @@
       <c r="E24" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="F24" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10446,7 +10460,7 @@
       <c r="E25" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10466,7 +10480,7 @@
       <c r="E26" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10486,7 +10500,7 @@
       <c r="E27" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F27" s="12" t="s">
+      <c r="F27" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10506,7 +10520,7 @@
       <c r="E28" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F28" s="12" t="s">
+      <c r="F28" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10526,6 +10540,7 @@
       <c r="E29" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F29" s="3"/>
     </row>
     <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -10543,6 +10558,7 @@
       <c r="E30" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F30" s="3"/>
     </row>
     <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
@@ -10560,6 +10576,7 @@
       <c r="E31" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
@@ -10577,6 +10594,7 @@
       <c r="E32" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F32" s="3"/>
     </row>
     <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
@@ -10594,6 +10612,7 @@
       <c r="E33" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F33" s="3"/>
     </row>
     <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
@@ -10611,6 +10630,7 @@
       <c r="E34" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F34" s="3"/>
     </row>
     <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
@@ -10628,6 +10648,7 @@
       <c r="E35" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F35" s="3"/>
     </row>
     <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
@@ -10645,6 +10666,7 @@
       <c r="E36" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F36" s="3"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
@@ -10662,7 +10684,7 @@
       <c r="E37" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F37" s="12" t="s">
+      <c r="F37" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10682,7 +10704,7 @@
       <c r="E38" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F38" s="12" t="s">
+      <c r="F38" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10702,7 +10724,7 @@
       <c r="E39" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F39" s="12" t="s">
+      <c r="F39" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10722,7 +10744,7 @@
       <c r="E40" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="F40" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10742,7 +10764,7 @@
       <c r="E41" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F41" s="12" t="s">
+      <c r="F41" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -10762,6 +10784,9 @@
       <c r="E42" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F42" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
@@ -10779,6 +10804,9 @@
       <c r="E43" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F43" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
@@ -10796,6 +10824,9 @@
       <c r="E44" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F44" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
@@ -10813,6 +10844,9 @@
       <c r="E45" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F45" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
@@ -10830,6 +10864,9 @@
       <c r="E46" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F46" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
@@ -10847,6 +10884,9 @@
       <c r="E47" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F47" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
@@ -10864,8 +10904,11 @@
       <c r="E48" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="4" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -10881,8 +10924,9 @@
       <c r="E49" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="3"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -10898,8 +10942,9 @@
       <c r="E50" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F50" s="3"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -10915,8 +10960,9 @@
       <c r="E51" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F51" s="3"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -10932,8 +10978,9 @@
       <c r="E52" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F52" s="3"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -10949,8 +10996,9 @@
       <c r="E53" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F53" s="3"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -10966,8 +11014,9 @@
       <c r="E54" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F54" s="3"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -10983,8 +11032,9 @@
       <c r="E55" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="3"/>
+    </row>
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -11000,8 +11050,9 @@
       <c r="E56" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F56" s="3"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -11017,8 +11068,9 @@
       <c r="E57" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" s="3"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -11034,8 +11086,9 @@
       <c r="E58" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F58" s="3"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -11051,8 +11104,9 @@
       <c r="E59" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" s="3"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -11068,8 +11122,9 @@
       <c r="E60" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F60" s="3"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -11085,8 +11140,9 @@
       <c r="E61" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" s="3"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -11102,8 +11158,9 @@
       <c r="E62" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F62" s="3"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -11119,8 +11176,9 @@
       <c r="E63" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" s="3"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -11136,6 +11194,7 @@
       <c r="E64" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F64" s="3"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
@@ -11153,6 +11212,7 @@
       <c r="E65" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F65" s="3"/>
     </row>
     <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
@@ -11170,6 +11230,7 @@
       <c r="E66" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F66" s="3"/>
     </row>
     <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
@@ -11187,6 +11248,7 @@
       <c r="E67" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F67" s="3"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
@@ -11204,7 +11266,7 @@
       <c r="E68" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F68" s="12" t="s">
+      <c r="F68" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -11224,7 +11286,7 @@
       <c r="E69" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F69" s="12" t="s">
+      <c r="F69" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -11244,7 +11306,7 @@
       <c r="E70" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F70" s="12" t="s">
+      <c r="F70" s="4" t="s">
         <v>514</v>
       </c>
     </row>
@@ -11264,6 +11326,9 @@
       <c r="E71" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F71" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
@@ -11281,6 +11346,9 @@
       <c r="E72" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F72" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
@@ -11298,6 +11366,9 @@
       <c r="E73" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F73" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
@@ -11315,6 +11386,7 @@
       <c r="E74" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F74" s="3"/>
     </row>
     <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
@@ -11332,6 +11404,7 @@
       <c r="E75" s="1" t="s">
         <v>456</v>
       </c>
+      <c r="F75" s="3"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
@@ -11349,6 +11422,7 @@
       <c r="E76" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F76" s="3"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
@@ -11366,6 +11440,7 @@
       <c r="E77" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F77" s="3"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
@@ -11383,6 +11458,7 @@
       <c r="E78" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F78" s="3"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
@@ -11400,6 +11476,7 @@
       <c r="E79" s="1" t="s">
         <v>455</v>
       </c>
+      <c r="F79" s="3"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
@@ -11417,8 +11494,9 @@
       <c r="E80" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F80" s="3"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -11434,8 +11512,9 @@
       <c r="E81" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F81" s="3"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -11451,8 +11530,9 @@
       <c r="E82" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F82" s="3"/>
+    </row>
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -11468,8 +11548,9 @@
       <c r="E83" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F83" s="3"/>
+    </row>
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -11485,8 +11566,9 @@
       <c r="E84" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F84" s="3"/>
+    </row>
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -11502,8 +11584,9 @@
       <c r="E85" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F85" s="3"/>
+    </row>
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -11519,8 +11602,9 @@
       <c r="E86" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F86" s="3"/>
+    </row>
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -11536,8 +11620,9 @@
       <c r="E87" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F87" s="3"/>
+    </row>
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -11553,8 +11638,9 @@
       <c r="E88" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F88" s="3"/>
+    </row>
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -11570,8 +11656,9 @@
       <c r="E89" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F89" s="3"/>
+    </row>
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -11587,8 +11674,9 @@
       <c r="E90" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F90" s="3"/>
+    </row>
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -11604,8 +11692,9 @@
       <c r="E91" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F91" s="3"/>
+    </row>
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -11621,8 +11710,9 @@
       <c r="E92" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F92" s="3"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -11638,8 +11728,9 @@
       <c r="E93" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F93" s="3"/>
+    </row>
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -11655,8 +11746,9 @@
       <c r="E94" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F94" s="3"/>
+    </row>
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -11672,8 +11764,9 @@
       <c r="E95" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F95" s="3"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -11689,8 +11782,9 @@
       <c r="E96" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F96" s="3"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -11706,8 +11800,9 @@
       <c r="E97" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F97" s="3"/>
+    </row>
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -11723,8 +11818,9 @@
       <c r="E98" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F98" s="3"/>
+    </row>
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -11740,8 +11836,9 @@
       <c r="E99" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F99" s="3"/>
+    </row>
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -11757,8 +11854,9 @@
       <c r="E100" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F100" s="3"/>
+    </row>
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -11774,8 +11872,9 @@
       <c r="E101" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F101" s="3"/>
+    </row>
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>101</v>
       </c>
@@ -11791,8 +11890,9 @@
       <c r="E102" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F102" s="3"/>
+    </row>
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>102</v>
       </c>
@@ -11808,8 +11908,9 @@
       <c r="E103" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F103" s="3"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>103</v>
       </c>
@@ -11825,8 +11926,9 @@
       <c r="E104" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F104" s="3"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>104</v>
       </c>
@@ -11842,8 +11944,9 @@
       <c r="E105" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F105" s="3"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>105</v>
       </c>
@@ -11859,8 +11962,9 @@
       <c r="E106" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F106" s="3"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>106</v>
       </c>
@@ -11876,8 +11980,9 @@
       <c r="E107" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F107" s="3"/>
+    </row>
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>107</v>
       </c>
@@ -11893,8 +11998,9 @@
       <c r="E108" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F108" s="3"/>
+    </row>
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>108</v>
       </c>
@@ -11910,8 +12016,9 @@
       <c r="E109" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F109" s="3"/>
+    </row>
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>109</v>
       </c>
@@ -11927,8 +12034,9 @@
       <c r="E110" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F110" s="3"/>
+    </row>
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>110</v>
       </c>
@@ -11944,8 +12052,9 @@
       <c r="E111" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F111" s="3"/>
+    </row>
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>111</v>
       </c>
@@ -11961,8 +12070,9 @@
       <c r="E112" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F112" s="3"/>
+    </row>
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>112</v>
       </c>
@@ -11978,8 +12088,9 @@
       <c r="E113" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F113" s="3"/>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>113</v>
       </c>
@@ -11995,8 +12106,9 @@
       <c r="E114" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F114" s="3"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>114</v>
       </c>
@@ -12012,8 +12124,9 @@
       <c r="E115" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F115" s="3"/>
+    </row>
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>115</v>
       </c>
@@ -12029,8 +12142,9 @@
       <c r="E116" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F116" s="3"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -12046,8 +12160,9 @@
       <c r="E117" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F117" s="3"/>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -12063,8 +12178,9 @@
       <c r="E118" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F118" s="3"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -12080,8 +12196,9 @@
       <c r="E119" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F119" s="3"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -12097,8 +12214,9 @@
       <c r="E120" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F120" s="3"/>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -12114,8 +12232,9 @@
       <c r="E121" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F121" s="3"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>121</v>
       </c>
@@ -12131,8 +12250,9 @@
       <c r="E122" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F122" s="3"/>
+    </row>
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>122</v>
       </c>
@@ -12148,8 +12268,9 @@
       <c r="E123" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F123" s="3"/>
+    </row>
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>123</v>
       </c>
@@ -12165,8 +12286,9 @@
       <c r="E124" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F124" s="3"/>
+    </row>
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>124</v>
       </c>
@@ -12182,8 +12304,9 @@
       <c r="E125" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F125" s="3"/>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>125</v>
       </c>
@@ -12199,8 +12322,9 @@
       <c r="E126" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F126" s="3"/>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>126</v>
       </c>
@@ -12216,8 +12340,9 @@
       <c r="E127" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F127" s="3"/>
+    </row>
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>127</v>
       </c>
@@ -12233,8 +12358,9 @@
       <c r="E128" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F128" s="3"/>
+    </row>
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>128</v>
       </c>
@@ -12250,8 +12376,9 @@
       <c r="E129" s="1" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F129" s="3"/>
+    </row>
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>129</v>
       </c>
@@ -12267,8 +12394,9 @@
       <c r="E130" s="1" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F130" s="3"/>
+    </row>
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>130</v>
       </c>
@@ -12284,8 +12412,9 @@
       <c r="E131" s="1" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F131" s="3"/>
+    </row>
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>131</v>
       </c>
@@ -12301,8 +12430,9 @@
       <c r="E132" s="1" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F132" s="3"/>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>132</v>
       </c>
@@ -12318,8 +12448,9 @@
       <c r="E133" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F133" s="3"/>
+    </row>
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>133</v>
       </c>
@@ -12335,8 +12466,9 @@
       <c r="E134" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F134" s="3"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>134</v>
       </c>
@@ -12352,8 +12484,9 @@
       <c r="E135" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F135" s="3"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>135</v>
       </c>
@@ -12369,8 +12502,9 @@
       <c r="E136" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F136" s="3"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>136</v>
       </c>
@@ -12386,8 +12520,9 @@
       <c r="E137" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F137" s="3"/>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>137</v>
       </c>
@@ -12403,8 +12538,9 @@
       <c r="E138" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F138" s="3"/>
+    </row>
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>138</v>
       </c>
@@ -12420,8 +12556,9 @@
       <c r="E139" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F139" s="3"/>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>139</v>
       </c>
@@ -12437,8 +12574,9 @@
       <c r="E140" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F140" s="3"/>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>140</v>
       </c>
@@ -12454,8 +12592,9 @@
       <c r="E141" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F141" s="3"/>
+    </row>
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>141</v>
       </c>
@@ -12471,8 +12610,9 @@
       <c r="E142" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F142" s="3"/>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>142</v>
       </c>
@@ -12488,8 +12628,9 @@
       <c r="E143" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F143" s="3"/>
+    </row>
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>143</v>
       </c>
@@ -12505,8 +12646,9 @@
       <c r="E144" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F144" s="3"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>144</v>
       </c>
@@ -12522,8 +12664,9 @@
       <c r="E145" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F145" s="3"/>
+    </row>
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>145</v>
       </c>
@@ -12539,8 +12682,9 @@
       <c r="E146" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F146" s="3"/>
+    </row>
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>146</v>
       </c>
@@ -12556,8 +12700,9 @@
       <c r="E147" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F147" s="3"/>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>147</v>
       </c>
@@ -12573,8 +12718,9 @@
       <c r="E148" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F148" s="3"/>
+    </row>
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>148</v>
       </c>
@@ -12590,8 +12736,9 @@
       <c r="E149" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F149" s="3"/>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>149</v>
       </c>
@@ -12607,8 +12754,9 @@
       <c r="E150" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F150" s="3"/>
+    </row>
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>150</v>
       </c>
@@ -12624,8 +12772,9 @@
       <c r="E151" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F151" s="3"/>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>151</v>
       </c>
@@ -12641,8 +12790,9 @@
       <c r="E152" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F152" s="3"/>
+    </row>
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>152</v>
       </c>
@@ -12658,8 +12808,9 @@
       <c r="E153" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F153" s="3"/>
+    </row>
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>153</v>
       </c>
@@ -12675,8 +12826,9 @@
       <c r="E154" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F154" s="3"/>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>154</v>
       </c>
@@ -12692,8 +12844,9 @@
       <c r="E155" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F155" s="3"/>
+    </row>
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>155</v>
       </c>
@@ -12709,8 +12862,9 @@
       <c r="E156" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F156" s="3"/>
+    </row>
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>156</v>
       </c>
@@ -12726,8 +12880,9 @@
       <c r="E157" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F157" s="3"/>
+    </row>
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>157</v>
       </c>
@@ -12743,8 +12898,9 @@
       <c r="E158" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F158" s="3"/>
+    </row>
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>158</v>
       </c>
@@ -12760,8 +12916,9 @@
       <c r="E159" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F159" s="3"/>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>159</v>
       </c>
@@ -12777,8 +12934,9 @@
       <c r="E160" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F160" s="3"/>
+    </row>
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>160</v>
       </c>
@@ -12794,8 +12952,9 @@
       <c r="E161" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F161" s="3"/>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>161</v>
       </c>
@@ -12811,8 +12970,9 @@
       <c r="E162" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F162" s="3"/>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>162</v>
       </c>
@@ -12828,8 +12988,9 @@
       <c r="E163" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F163" s="3"/>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>163</v>
       </c>
@@ -12845,8 +13006,9 @@
       <c r="E164" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F164" s="3"/>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>164</v>
       </c>
@@ -12862,8 +13024,9 @@
       <c r="E165" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F165" s="3"/>
+    </row>
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>165</v>
       </c>
@@ -12879,8 +13042,9 @@
       <c r="E166" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F166" s="3"/>
+    </row>
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>166</v>
       </c>
@@ -12896,8 +13060,9 @@
       <c r="E167" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F167" s="3"/>
+    </row>
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>167</v>
       </c>
@@ -12913,8 +13078,9 @@
       <c r="E168" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F168" s="3"/>
+    </row>
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>168</v>
       </c>
@@ -12930,8 +13096,9 @@
       <c r="E169" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F169" s="3"/>
+    </row>
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>169</v>
       </c>
@@ -12947,8 +13114,9 @@
       <c r="E170" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F170" s="3"/>
+    </row>
+    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>170</v>
       </c>
@@ -12964,8 +13132,9 @@
       <c r="E171" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F171" s="3"/>
+    </row>
+    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>171</v>
       </c>
@@ -12981,8 +13150,9 @@
       <c r="E172" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F172" s="3"/>
+    </row>
+    <row r="173" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>172</v>
       </c>
@@ -12998,8 +13168,9 @@
       <c r="E173" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F173" s="3"/>
+    </row>
+    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>173</v>
       </c>
@@ -13015,8 +13186,9 @@
       <c r="E174" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F174" s="3"/>
+    </row>
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>174</v>
       </c>
@@ -13032,8 +13204,9 @@
       <c r="E175" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F175" s="3"/>
+    </row>
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>175</v>
       </c>
@@ -13049,8 +13222,9 @@
       <c r="E176" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F176" s="3"/>
+    </row>
+    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="1">
         <v>176</v>
       </c>
@@ -13066,8 +13240,9 @@
       <c r="E177" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F177" s="3"/>
+    </row>
+    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="1">
         <v>177</v>
       </c>
@@ -13083,8 +13258,9 @@
       <c r="E178" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F178" s="3"/>
+    </row>
+    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="1">
         <v>178</v>
       </c>
@@ -13100,8 +13276,9 @@
       <c r="E179" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F179" s="3"/>
+    </row>
+    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="1">
         <v>179</v>
       </c>
@@ -13117,8 +13294,9 @@
       <c r="E180" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F180" s="3"/>
+    </row>
+    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="1">
         <v>180</v>
       </c>
@@ -13134,8 +13312,9 @@
       <c r="E181" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F181" s="3"/>
+    </row>
+    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="1">
         <v>181</v>
       </c>
@@ -13151,8 +13330,9 @@
       <c r="E182" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F182" s="3"/>
+    </row>
+    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="1">
         <v>182</v>
       </c>
@@ -13168,8 +13348,9 @@
       <c r="E183" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F183" s="3"/>
+    </row>
+    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="1">
         <v>183</v>
       </c>
@@ -13185,8 +13366,9 @@
       <c r="E184" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F184" s="3"/>
+    </row>
+    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="1">
         <v>184</v>
       </c>
@@ -13202,8 +13384,9 @@
       <c r="E185" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F185" s="3"/>
+    </row>
+    <row r="186" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="1">
         <v>185</v>
       </c>
@@ -13219,8 +13402,9 @@
       <c r="E186" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F186" s="3"/>
+    </row>
+    <row r="187" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="1">
         <v>186</v>
       </c>
@@ -13236,8 +13420,9 @@
       <c r="E187" s="1" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F187" s="3"/>
+    </row>
+    <row r="188" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="1">
         <v>187</v>
       </c>
@@ -13253,8 +13438,9 @@
       <c r="E188" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F188" s="3"/>
+    </row>
+    <row r="189" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="1">
         <v>188</v>
       </c>
@@ -13270,8 +13456,9 @@
       <c r="E189" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F189" s="3"/>
+    </row>
+    <row r="190" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="1">
         <v>189</v>
       </c>
@@ -13287,8 +13474,9 @@
       <c r="E190" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F190" s="3"/>
+    </row>
+    <row r="191" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="1">
         <v>190</v>
       </c>
@@ -13304,8 +13492,9 @@
       <c r="E191" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F191" s="3"/>
+    </row>
+    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="1">
         <v>191</v>
       </c>
@@ -13321,8 +13510,9 @@
       <c r="E192" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F192" s="3"/>
+    </row>
+    <row r="193" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="1">
         <v>192</v>
       </c>
@@ -13338,8 +13528,9 @@
       <c r="E193" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F193" s="3"/>
+    </row>
+    <row r="194" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="1">
         <v>193</v>
       </c>
@@ -13355,8 +13546,9 @@
       <c r="E194" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F194" s="3"/>
+    </row>
+    <row r="195" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="1">
         <v>194</v>
       </c>
@@ -13372,8 +13564,9 @@
       <c r="E195" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F195" s="3"/>
+    </row>
+    <row r="196" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="1">
         <v>195</v>
       </c>
@@ -13389,8 +13582,9 @@
       <c r="E196" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F196" s="3"/>
+    </row>
+    <row r="197" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="1">
         <v>196</v>
       </c>
@@ -13406,8 +13600,9 @@
       <c r="E197" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F197" s="3"/>
+    </row>
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="1">
         <v>197</v>
       </c>
@@ -13423,8 +13618,9 @@
       <c r="E198" s="1" t="s">
         <v>458</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F198" s="3"/>
+    </row>
+    <row r="199" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="1">
         <v>198</v>
       </c>
@@ -13440,8 +13636,9 @@
       <c r="E199" s="1" t="s">
         <v>457</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F199" s="3"/>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>199</v>
       </c>
@@ -13457,18 +13654,19 @@
       <c r="E200" s="1" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F200" s="3"/>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B205" s="11" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B206" s="11" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B207" s="11" t="s">
         <v>513</v>
       </c>
@@ -13495,12 +13693,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>515</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>516</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added few topics in java 50
</commit_message>
<xml_diff>
--- a/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
+++ b/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2737" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="517">
   <si>
     <t>Category</t>
   </si>
@@ -10924,7 +10924,9 @@
       <c r="E49" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F49" s="3"/>
+      <c r="F49" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
@@ -10942,7 +10944,9 @@
       <c r="E50" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F50" s="3"/>
+      <c r="F50" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
@@ -10960,7 +10964,9 @@
       <c r="E51" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F51" s="3"/>
+      <c r="F51" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
@@ -10978,7 +10984,9 @@
       <c r="E52" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F52" s="3"/>
+      <c r="F52" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
@@ -10996,7 +11004,9 @@
       <c r="E53" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F53" s="3"/>
+      <c r="F53" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
@@ -11014,7 +11024,9 @@
       <c r="E54" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F54" s="3"/>
+      <c r="F54" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
@@ -11032,7 +11044,9 @@
       <c r="E55" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F55" s="3"/>
+      <c r="F55" s="4" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
@@ -12936,7 +12950,7 @@
       </c>
       <c r="F160" s="3"/>
     </row>
-    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>160</v>
       </c>
@@ -12950,7 +12964,7 @@
         <v>389</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F161" s="3"/>
     </row>

</xml_diff>

<commit_message>
p1 added for java 50
</commit_message>
<xml_diff>
--- a/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
+++ b/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2755" uniqueCount="517">
   <si>
     <t>Category</t>
   </si>
@@ -1563,9 +1563,6 @@
     <t xml:space="preserve"> 2) 50 question and answer of interview theory</t>
   </si>
   <si>
-    <t>3) 50 coding practical question and answer interview coding round</t>
-  </si>
-  <si>
     <t>Complete</t>
   </si>
   <si>
@@ -1573,6 +1570,9 @@
   </si>
   <si>
     <t>https://wissen.zohorecruit.in/jobs/Careers/80238000057776296/Java-Lead?source=LinkedIn-Premium&amp;embedsource=LinkedIn%2BLimited%2BListings</t>
+  </si>
+  <si>
+    <t>3)6 coding practical question and answer interview coding round</t>
   </si>
 </sst>
 </file>
@@ -10145,7 +10145,7 @@
         <v>455</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -10165,7 +10165,7 @@
         <v>455</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -10203,7 +10203,7 @@
         <v>455</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -10223,7 +10223,7 @@
         <v>455</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -10243,7 +10243,7 @@
         <v>455</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -10281,7 +10281,7 @@
         <v>455</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -10301,7 +10301,7 @@
         <v>455</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -10321,7 +10321,7 @@
         <v>455</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -10341,7 +10341,7 @@
         <v>455</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -10361,7 +10361,7 @@
         <v>455</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -10381,7 +10381,7 @@
         <v>455</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -10401,7 +10401,7 @@
         <v>455</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -10421,7 +10421,7 @@
         <v>455</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -10441,7 +10441,7 @@
         <v>455</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -10461,7 +10461,7 @@
         <v>455</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -10481,7 +10481,7 @@
         <v>455</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -10501,7 +10501,7 @@
         <v>455</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -10521,7 +10521,7 @@
         <v>455</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -10685,7 +10685,7 @@
         <v>455</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -10705,7 +10705,7 @@
         <v>455</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -10725,7 +10725,7 @@
         <v>455</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -10745,7 +10745,7 @@
         <v>455</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -10765,7 +10765,7 @@
         <v>455</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -10785,7 +10785,7 @@
         <v>455</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -10805,7 +10805,7 @@
         <v>455</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -10825,7 +10825,7 @@
         <v>455</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -10845,7 +10845,7 @@
         <v>455</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -10865,7 +10865,7 @@
         <v>455</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -10885,7 +10885,7 @@
         <v>455</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -10905,7 +10905,7 @@
         <v>455</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -10925,7 +10925,7 @@
         <v>455</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -10945,7 +10945,7 @@
         <v>455</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -10965,7 +10965,7 @@
         <v>455</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -10985,7 +10985,7 @@
         <v>455</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -11005,7 +11005,7 @@
         <v>455</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -11025,7 +11025,7 @@
         <v>455</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -11045,7 +11045,7 @@
         <v>455</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -11082,7 +11082,9 @@
       <c r="E57" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F57" s="3"/>
+      <c r="F57" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
@@ -11100,7 +11102,9 @@
       <c r="E58" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F58" s="3"/>
+      <c r="F58" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
@@ -11118,7 +11122,9 @@
       <c r="E59" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F59" s="3"/>
+      <c r="F59" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
@@ -11136,7 +11142,9 @@
       <c r="E60" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F60" s="3"/>
+      <c r="F60" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
@@ -11154,7 +11162,9 @@
       <c r="E61" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F61" s="3"/>
+      <c r="F61" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
@@ -11172,7 +11182,9 @@
       <c r="E62" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F62" s="3"/>
+      <c r="F62" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
@@ -11190,7 +11202,9 @@
       <c r="E63" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F63" s="3"/>
+      <c r="F63" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
@@ -11208,7 +11222,9 @@
       <c r="E64" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F64" s="3"/>
+      <c r="F64" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
@@ -11226,9 +11242,11 @@
       <c r="E65" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F65" s="3"/>
-    </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F65" s="4" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -11242,11 +11260,13 @@
         <v>202</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="F66" s="3"/>
-    </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -11260,9 +11280,11 @@
         <v>204</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="F67" s="3"/>
+        <v>455</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
@@ -11281,7 +11303,7 @@
         <v>455</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -11301,7 +11323,7 @@
         <v>455</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -11321,7 +11343,7 @@
         <v>455</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -11341,7 +11363,7 @@
         <v>455</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -11361,7 +11383,7 @@
         <v>455</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -11381,7 +11403,7 @@
         <v>455</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -11816,7 +11838,7 @@
       </c>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -11830,11 +11852,11 @@
         <v>258</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -11848,11 +11870,11 @@
         <v>260</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -11866,7 +11888,7 @@
         <v>262</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F100" s="3"/>
     </row>
@@ -12140,7 +12162,7 @@
       </c>
       <c r="F115" s="3"/>
     </row>
-    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>115</v>
       </c>
@@ -12154,7 +12176,7 @@
         <v>32</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F116" s="3"/>
     </row>
@@ -12356,7 +12378,7 @@
       </c>
       <c r="F127" s="3"/>
     </row>
-    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>127</v>
       </c>
@@ -12370,7 +12392,7 @@
         <v>322</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F128" s="3"/>
     </row>
@@ -13682,7 +13704,7 @@
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B207" s="11" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
   </sheetData>
@@ -13708,12 +13730,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added core java quieck interview
</commit_message>
<xml_diff>
--- a/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
+++ b/TheorynCoding/Study Material/Java Overall/Java Topics Overview.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,7 @@
     <sheet name="Sheet2" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="6" r:id="rId4"/>
     <sheet name="Sheet4" sheetId="7" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="8" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet3!$A$1:$G$199</definedName>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2713" uniqueCount="528">
   <si>
     <t>Category</t>
   </si>
@@ -1603,13 +1604,16 @@
   </si>
   <si>
     <t>inprogress</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/java/difference-between-spring-boot-starter-web-and-spring-boot-starter-tomcat/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1628,6 +1632,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1682,10 +1694,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1722,8 +1735,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -10032,7 +10047,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -10050,7 +10065,7 @@
       </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -10068,7 +10083,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -10086,7 +10101,7 @@
       </c>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -10104,7 +10119,7 @@
       </c>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -10122,7 +10137,7 @@
       </c>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -10140,7 +10155,7 @@
       </c>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -10158,7 +10173,7 @@
       </c>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -10178,7 +10193,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -10196,7 +10211,7 @@
       </c>
       <c r="F10" s="4"/>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -10214,7 +10229,7 @@
       </c>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -10232,7 +10247,7 @@
       </c>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -10250,7 +10265,7 @@
       </c>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -10268,7 +10283,7 @@
       </c>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -10286,7 +10301,7 @@
       </c>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -10304,7 +10319,7 @@
       </c>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -10322,7 +10337,7 @@
       </c>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -10340,7 +10355,7 @@
       </c>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -10358,7 +10373,7 @@
       </c>
       <c r="F19" s="4"/>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -10374,11 +10389,9 @@
       <c r="E20" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="4"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -10394,11 +10407,9 @@
       <c r="E21" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -10414,11 +10425,9 @@
       <c r="E22" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F22" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="4"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -10434,11 +10443,9 @@
       <c r="E23" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -10454,11 +10461,9 @@
       <c r="E24" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -10474,11 +10479,9 @@
       <c r="E25" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F25" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -10494,11 +10497,9 @@
       <c r="E26" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F26" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -10514,11 +10515,9 @@
       <c r="E27" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -10534,11 +10533,9 @@
       <c r="E28" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -10554,11 +10551,9 @@
       <c r="E29" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -10574,11 +10569,9 @@
       <c r="E30" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F30" s="4"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -10594,11 +10587,9 @@
       <c r="E31" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -10614,11 +10605,9 @@
       <c r="E32" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -10634,11 +10623,9 @@
       <c r="E33" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F33" s="4"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -10654,11 +10641,9 @@
       <c r="E34" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -10674,11 +10659,9 @@
       <c r="E35" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -10694,11 +10677,9 @@
       <c r="E36" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -10716,7 +10697,7 @@
       </c>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -10734,7 +10715,7 @@
       </c>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -10752,7 +10733,7 @@
       </c>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -10770,7 +10751,7 @@
       </c>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -10788,7 +10769,7 @@
       </c>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -10804,11 +10785,9 @@
       <c r="E42" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F42" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F42" s="4"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -10824,11 +10803,9 @@
       <c r="E43" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F43" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F43" s="4"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -10844,11 +10821,9 @@
       <c r="E44" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F44" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F44" s="4"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -10864,11 +10839,9 @@
       <c r="E45" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F45" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F45" s="4"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -10884,11 +10857,9 @@
       <c r="E46" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F46" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -10904,11 +10875,9 @@
       <c r="E47" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F47" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F47" s="4"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -10924,11 +10893,9 @@
       <c r="E48" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F48" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F48" s="4"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -10944,11 +10911,9 @@
       <c r="E49" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F49" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F49" s="4"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -10964,11 +10929,9 @@
       <c r="E50" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F50" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -10984,11 +10947,9 @@
       <c r="E51" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F51" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F51" s="4"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -11004,11 +10965,9 @@
       <c r="E52" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F52" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F52" s="4"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -11024,11 +10983,9 @@
       <c r="E53" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F53" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F53" s="4"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -11044,11 +11001,9 @@
       <c r="E54" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F54" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F54" s="4"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -11064,11 +11019,9 @@
       <c r="E55" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="F55" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="4"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -11084,11 +11037,9 @@
       <c r="E56" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="F56" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F56" s="4"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -11106,7 +11057,7 @@
       </c>
       <c r="F57" s="4"/>
     </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -11124,7 +11075,7 @@
       </c>
       <c r="F58" s="4"/>
     </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -11142,7 +11093,7 @@
       </c>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -11160,7 +11111,7 @@
       </c>
       <c r="F60" s="4"/>
     </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -11178,7 +11129,7 @@
       </c>
       <c r="F61" s="4"/>
     </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -11196,7 +11147,7 @@
       </c>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -11214,7 +11165,7 @@
       </c>
       <c r="F63" s="4"/>
     </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -11232,7 +11183,7 @@
       </c>
       <c r="F64" s="4"/>
     </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -11250,7 +11201,7 @@
       </c>
       <c r="F65" s="4"/>
     </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -11268,7 +11219,7 @@
       </c>
       <c r="F66" s="4"/>
     </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -11286,7 +11237,7 @@
       </c>
       <c r="F67" s="4"/>
     </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -11304,7 +11255,7 @@
       </c>
       <c r="F68" s="4"/>
     </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -11322,7 +11273,7 @@
       </c>
       <c r="F69" s="4"/>
     </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -11340,7 +11291,7 @@
       </c>
       <c r="F70" s="4"/>
     </row>
-    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -11358,7 +11309,7 @@
       </c>
       <c r="F71" s="4"/>
     </row>
-    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -11376,7 +11327,7 @@
       </c>
       <c r="F72" s="4"/>
     </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -11394,7 +11345,7 @@
       </c>
       <c r="F73" s="4"/>
     </row>
-    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -11412,7 +11363,7 @@
       </c>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -11430,7 +11381,7 @@
       </c>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -11448,7 +11399,7 @@
       </c>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -11466,7 +11417,7 @@
       </c>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -11484,7 +11435,7 @@
       </c>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -11502,7 +11453,7 @@
       </c>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -11520,7 +11471,7 @@
       </c>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -11538,7 +11489,7 @@
       </c>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -11556,12 +11507,12 @@
       </c>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>10</v>
@@ -11574,12 +11525,12 @@
       </c>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>10</v>
@@ -11592,12 +11543,12 @@
       </c>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>10</v>
@@ -11610,12 +11561,12 @@
       </c>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>10</v>
@@ -11628,12 +11579,12 @@
       </c>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>10</v>
@@ -11646,12 +11597,12 @@
       </c>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>10</v>
@@ -11664,12 +11615,12 @@
       </c>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>232</v>
@@ -11682,12 +11633,12 @@
       </c>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>232</v>
@@ -11700,12 +11651,12 @@
       </c>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>11</v>
@@ -11718,12 +11669,12 @@
       </c>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>1</v>
+        <v>232</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>11</v>
@@ -11736,12 +11687,12 @@
       </c>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>13</v>
@@ -11754,12 +11705,12 @@
       </c>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>13</v>
@@ -11772,12 +11723,12 @@
       </c>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>13</v>
@@ -11790,12 +11741,12 @@
       </c>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>253</v>
@@ -11808,12 +11759,12 @@
       </c>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>253</v>
@@ -11826,12 +11777,12 @@
       </c>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>253</v>
@@ -11844,12 +11795,12 @@
       </c>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>253</v>
@@ -11862,12 +11813,12 @@
       </c>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>253</v>
@@ -11880,12 +11831,12 @@
       </c>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>1</v>
+        <v>281</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>281</v>
@@ -11898,12 +11849,12 @@
       </c>
       <c r="F101" s="3"/>
     </row>
-    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>1</v>
+        <v>281</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>281</v>
@@ -11916,12 +11867,12 @@
       </c>
       <c r="F102" s="3"/>
     </row>
-    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>1</v>
+        <v>281</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>281</v>
@@ -11934,7 +11885,7 @@
       </c>
       <c r="F103" s="3"/>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>103</v>
       </c>
@@ -11952,7 +11903,7 @@
       </c>
       <c r="F104" s="3"/>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>104</v>
       </c>
@@ -11970,7 +11921,7 @@
       </c>
       <c r="F105" s="3"/>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>105</v>
       </c>
@@ -11988,7 +11939,7 @@
       </c>
       <c r="F106" s="3"/>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>106</v>
       </c>
@@ -12006,7 +11957,7 @@
       </c>
       <c r="F107" s="3"/>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>107</v>
       </c>
@@ -12024,7 +11975,7 @@
       </c>
       <c r="F108" s="3"/>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>108</v>
       </c>
@@ -12042,7 +11993,7 @@
       </c>
       <c r="F109" s="3"/>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>109</v>
       </c>
@@ -12060,7 +12011,7 @@
       </c>
       <c r="F110" s="3"/>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>110</v>
       </c>
@@ -12078,7 +12029,7 @@
       </c>
       <c r="F111" s="3"/>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>111</v>
       </c>
@@ -12096,7 +12047,7 @@
       </c>
       <c r="F112" s="3"/>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>112</v>
       </c>
@@ -12114,7 +12065,7 @@
       </c>
       <c r="F113" s="3"/>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>113</v>
       </c>
@@ -12132,7 +12083,7 @@
       </c>
       <c r="F114" s="3"/>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>114</v>
       </c>
@@ -12150,7 +12101,7 @@
       </c>
       <c r="F115" s="3"/>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>115</v>
       </c>
@@ -12168,7 +12119,7 @@
       </c>
       <c r="F116" s="3"/>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -12186,7 +12137,7 @@
       </c>
       <c r="F117" s="3"/>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -12206,7 +12157,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -12224,7 +12175,7 @@
       </c>
       <c r="F119" s="3"/>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -12242,7 +12193,7 @@
       </c>
       <c r="F120" s="3"/>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -12260,7 +12211,7 @@
       </c>
       <c r="F121" s="3"/>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>121</v>
       </c>
@@ -12278,7 +12229,7 @@
       </c>
       <c r="F122" s="3"/>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>122</v>
       </c>
@@ -12296,7 +12247,7 @@
       </c>
       <c r="F123" s="3"/>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>123</v>
       </c>
@@ -12314,7 +12265,7 @@
       </c>
       <c r="F124" s="3"/>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>124</v>
       </c>
@@ -12332,7 +12283,7 @@
       </c>
       <c r="F125" s="3"/>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>125</v>
       </c>
@@ -12350,7 +12301,7 @@
       </c>
       <c r="F126" s="3"/>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>126</v>
       </c>
@@ -12368,7 +12319,7 @@
       </c>
       <c r="F127" s="3"/>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>127</v>
       </c>
@@ -12386,7 +12337,7 @@
       </c>
       <c r="F128" s="3"/>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>128</v>
       </c>
@@ -12404,7 +12355,7 @@
       </c>
       <c r="F129" s="3"/>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>129</v>
       </c>
@@ -12422,7 +12373,7 @@
       </c>
       <c r="F130" s="3"/>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>130</v>
       </c>
@@ -12440,7 +12391,7 @@
       </c>
       <c r="F131" s="3"/>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>131</v>
       </c>
@@ -12458,7 +12409,7 @@
       </c>
       <c r="F132" s="3"/>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>132</v>
       </c>
@@ -12476,7 +12427,7 @@
       </c>
       <c r="F133" s="3"/>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>133</v>
       </c>
@@ -12494,7 +12445,7 @@
       </c>
       <c r="F134" s="3"/>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>134</v>
       </c>
@@ -12512,7 +12463,7 @@
       </c>
       <c r="F135" s="3"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>135</v>
       </c>
@@ -12530,7 +12481,7 @@
       </c>
       <c r="F136" s="3"/>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>136</v>
       </c>
@@ -12548,7 +12499,7 @@
       </c>
       <c r="F137" s="3"/>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>137</v>
       </c>
@@ -12566,7 +12517,7 @@
       </c>
       <c r="F138" s="3"/>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>138</v>
       </c>
@@ -12584,7 +12535,7 @@
       </c>
       <c r="F139" s="3"/>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>139</v>
       </c>
@@ -12602,7 +12553,7 @@
       </c>
       <c r="F140" s="3"/>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>140</v>
       </c>
@@ -12620,7 +12571,7 @@
       </c>
       <c r="F141" s="3"/>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>141</v>
       </c>
@@ -12638,7 +12589,7 @@
       </c>
       <c r="F142" s="3"/>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>142</v>
       </c>
@@ -12656,7 +12607,7 @@
       </c>
       <c r="F143" s="3"/>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>143</v>
       </c>
@@ -12674,7 +12625,7 @@
       </c>
       <c r="F144" s="3"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>144</v>
       </c>
@@ -12692,7 +12643,7 @@
       </c>
       <c r="F145" s="3"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>145</v>
       </c>
@@ -12710,7 +12661,7 @@
       </c>
       <c r="F146" s="3"/>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>146</v>
       </c>
@@ -12728,7 +12679,7 @@
       </c>
       <c r="F147" s="3"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>147</v>
       </c>
@@ -12746,7 +12697,7 @@
       </c>
       <c r="F148" s="3"/>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>148</v>
       </c>
@@ -12764,7 +12715,7 @@
       </c>
       <c r="F149" s="3"/>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>149</v>
       </c>
@@ -12782,7 +12733,7 @@
       </c>
       <c r="F150" s="3"/>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>150</v>
       </c>
@@ -12800,7 +12751,7 @@
       </c>
       <c r="F151" s="3"/>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>151</v>
       </c>
@@ -12818,7 +12769,7 @@
       </c>
       <c r="F152" s="3"/>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>152</v>
       </c>
@@ -12836,7 +12787,7 @@
       </c>
       <c r="F153" s="3"/>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>153</v>
       </c>
@@ -12854,7 +12805,7 @@
       </c>
       <c r="F154" s="3"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>154</v>
       </c>
@@ -12872,7 +12823,7 @@
       </c>
       <c r="F155" s="3"/>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>155</v>
       </c>
@@ -12890,7 +12841,7 @@
       </c>
       <c r="F156" s="3"/>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>156</v>
       </c>
@@ -12908,7 +12859,7 @@
       </c>
       <c r="F157" s="3"/>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>157</v>
       </c>
@@ -12926,7 +12877,7 @@
       </c>
       <c r="F158" s="3"/>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>158</v>
       </c>
@@ -12944,7 +12895,7 @@
       </c>
       <c r="F159" s="3"/>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>159</v>
       </c>
@@ -12962,7 +12913,7 @@
       </c>
       <c r="F160" s="3"/>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>160</v>
       </c>
@@ -13664,7 +13615,7 @@
       </c>
       <c r="F199" s="3"/>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="1">
         <v>199</v>
       </c>
@@ -13746,7 +13697,7 @@
   <autoFilter ref="A1:F200">
     <filterColumn colId="1">
       <filters>
-        <filter val="Advanced Java"/>
+        <filter val="Core Java"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -13776,4 +13727,25 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="107.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>527</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>